<commit_message>
add html_cleaner.py for post-processing HTML files. Update README to include instructions for using the new cleaning script.
</commit_message>
<xml_diff>
--- a/metrics/evaluation/gemini_correctness_report.xlsx
+++ b/metrics/evaluation/gemini_correctness_report.xlsx
@@ -783,13 +783,13 @@
         <v>1</v>
       </c>
       <c r="C15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -879,13 +879,13 @@
         <v>1</v>
       </c>
       <c r="C19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -927,13 +927,13 @@
         <v>1</v>
       </c>
       <c r="C21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -951,13 +951,13 @@
         <v>1</v>
       </c>
       <c r="C22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1239,13 +1239,13 @@
         <v>1</v>
       </c>
       <c r="C34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1455,13 +1455,13 @@
         <v>1</v>
       </c>
       <c r="C43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1527,13 +1527,13 @@
         <v>1</v>
       </c>
       <c r="C46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1575,13 +1575,13 @@
         <v>1</v>
       </c>
       <c r="C48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -1719,13 +1719,13 @@
         <v>1</v>
       </c>
       <c r="C54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54" t="n">
         <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1959,13 +1959,13 @@
         <v>1</v>
       </c>
       <c r="C64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" t="n">
         <v>0</v>
       </c>
       <c r="E64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2151,13 +2151,13 @@
         <v>1</v>
       </c>
       <c r="C72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72" t="n">
         <v>0</v>
       </c>
       <c r="E72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2223,13 +2223,13 @@
         <v>1</v>
       </c>
       <c r="C75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
         <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -2463,13 +2463,13 @@
         <v>1</v>
       </c>
       <c r="C85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D85" t="n">
         <v>0</v>
       </c>
       <c r="E85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -2703,13 +2703,13 @@
         <v>1</v>
       </c>
       <c r="C95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95" t="n">
         <v>0</v>
       </c>
       <c r="E95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -2799,13 +2799,13 @@
         <v>1</v>
       </c>
       <c r="C99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D99" t="n">
         <v>0</v>
       </c>
       <c r="E99" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -2847,13 +2847,13 @@
         <v>1</v>
       </c>
       <c r="C101" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D101" t="n">
         <v>0</v>
       </c>
       <c r="E101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -2871,13 +2871,13 @@
         <v>1</v>
       </c>
       <c r="C102" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D102" t="n">
         <v>0</v>
       </c>
       <c r="E102" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -2895,13 +2895,13 @@
         <v>1</v>
       </c>
       <c r="C103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D103" t="n">
         <v>0</v>
       </c>
       <c r="E103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -3039,13 +3039,13 @@
         <v>1</v>
       </c>
       <c r="C109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D109" t="n">
         <v>0</v>
       </c>
       <c r="E109" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3063,13 +3063,13 @@
         <v>1</v>
       </c>
       <c r="C110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D110" t="n">
         <v>0</v>
       </c>
       <c r="E110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3207,13 +3207,13 @@
         <v>1</v>
       </c>
       <c r="C116" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D116" t="n">
         <v>0</v>
       </c>
       <c r="E116" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
@@ -3279,13 +3279,13 @@
         <v>1</v>
       </c>
       <c r="C119" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D119" t="n">
         <v>0</v>
       </c>
       <c r="E119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -3615,13 +3615,13 @@
         <v>1</v>
       </c>
       <c r="C133" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D133" t="n">
         <v>0</v>
       </c>
       <c r="E133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -3831,13 +3831,13 @@
         <v>1</v>
       </c>
       <c r="C142" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D142" t="n">
         <v>0</v>
       </c>
       <c r="E142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -3855,13 +3855,13 @@
         <v>1</v>
       </c>
       <c r="C143" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D143" t="n">
         <v>0</v>
       </c>
       <c r="E143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
@@ -4095,13 +4095,13 @@
         <v>1</v>
       </c>
       <c r="C153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D153" t="n">
         <v>0</v>
       </c>
       <c r="E153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -4119,13 +4119,13 @@
         <v>1</v>
       </c>
       <c r="C154" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D154" t="n">
         <v>0</v>
       </c>
       <c r="E154" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -4143,13 +4143,13 @@
         <v>1</v>
       </c>
       <c r="C155" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D155" t="n">
         <v>0</v>
       </c>
       <c r="E155" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -4191,13 +4191,13 @@
         <v>1</v>
       </c>
       <c r="C157" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D157" t="n">
         <v>0</v>
       </c>
       <c r="E157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -4239,13 +4239,13 @@
         <v>1</v>
       </c>
       <c r="C159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D159" t="n">
         <v>0</v>
       </c>
       <c r="E159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -4359,13 +4359,13 @@
         <v>1</v>
       </c>
       <c r="C164" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D164" t="n">
         <v>0</v>
       </c>
       <c r="E164" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F164" t="inlineStr">
         <is>
@@ -4383,13 +4383,13 @@
         <v>1</v>
       </c>
       <c r="C165" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D165" t="n">
         <v>0</v>
       </c>
       <c r="E165" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F165" t="inlineStr">
         <is>
@@ -4407,13 +4407,13 @@
         <v>1</v>
       </c>
       <c r="C166" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D166" t="n">
         <v>0</v>
       </c>
       <c r="E166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F166" t="inlineStr">
         <is>
@@ -4599,13 +4599,13 @@
         <v>1</v>
       </c>
       <c r="C174" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D174" t="n">
         <v>0</v>
       </c>
       <c r="E174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F174" t="inlineStr">
         <is>
@@ -4743,13 +4743,13 @@
         <v>1</v>
       </c>
       <c r="C180" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D180" t="n">
         <v>0</v>
       </c>
       <c r="E180" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F180" t="inlineStr">
         <is>
@@ -4791,13 +4791,13 @@
         <v>1</v>
       </c>
       <c r="C182" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D182" t="n">
         <v>0</v>
       </c>
       <c r="E182" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F182" t="inlineStr">
         <is>
@@ -4887,13 +4887,13 @@
         <v>1</v>
       </c>
       <c r="C186" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D186" t="n">
         <v>0</v>
       </c>
       <c r="E186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F186" t="inlineStr">
         <is>
@@ -4959,13 +4959,13 @@
         <v>1</v>
       </c>
       <c r="C189" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D189" t="n">
         <v>0</v>
       </c>
       <c r="E189" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F189" t="inlineStr">
         <is>
@@ -5007,13 +5007,13 @@
         <v>1</v>
       </c>
       <c r="C191" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D191" t="n">
         <v>0</v>
       </c>
       <c r="E191" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F191" t="inlineStr">
         <is>
@@ -5127,13 +5127,13 @@
         <v>1</v>
       </c>
       <c r="C196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D196" t="n">
         <v>0</v>
       </c>
       <c r="E196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F196" t="inlineStr">
         <is>
@@ -5175,13 +5175,13 @@
         <v>1</v>
       </c>
       <c r="C198" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D198" t="n">
         <v>0</v>
       </c>
       <c r="E198" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F198" t="inlineStr">
         <is>
@@ -5751,13 +5751,13 @@
         <v>1</v>
       </c>
       <c r="C222" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D222" t="n">
         <v>0</v>
       </c>
       <c r="E222" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F222" t="inlineStr">
         <is>
@@ -5874,14 +5874,14 @@
         <v>1</v>
       </c>
       <c r="D227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E227" t="n">
         <v>0</v>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>['[Console Error]: Failed to load resource: net::ERR_FILE_NOT_FOUND']</t>
+          <t>['[Console Error]: Failed to load resource: net::ERR_FILE_NOT_FOUND', '[Console Error]: Failed to load resource: net::ERR_FILE_NOT_FOUND']</t>
         </is>
       </c>
     </row>
@@ -5919,13 +5919,13 @@
         <v>1</v>
       </c>
       <c r="C229" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D229" t="n">
         <v>0</v>
       </c>
       <c r="E229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F229" t="inlineStr">
         <is>
@@ -5943,13 +5943,13 @@
         <v>1</v>
       </c>
       <c r="C230" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D230" t="n">
         <v>0</v>
       </c>
       <c r="E230" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F230" t="inlineStr">
         <is>
@@ -6015,13 +6015,13 @@
         <v>1</v>
       </c>
       <c r="C233" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" t="n">
         <v>0</v>
       </c>
       <c r="E233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F233" t="inlineStr">
         <is>
@@ -6039,13 +6039,13 @@
         <v>1</v>
       </c>
       <c r="C234" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D234" t="n">
         <v>0</v>
       </c>
       <c r="E234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F234" t="inlineStr">
         <is>
@@ -6279,13 +6279,13 @@
         <v>1</v>
       </c>
       <c r="C244" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D244" t="n">
         <v>0</v>
       </c>
       <c r="E244" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F244" t="inlineStr">
         <is>
@@ -6495,13 +6495,13 @@
         <v>1</v>
       </c>
       <c r="C253" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D253" t="n">
         <v>0</v>
       </c>
       <c r="E253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F253" t="inlineStr">
         <is>
@@ -6639,13 +6639,13 @@
         <v>1</v>
       </c>
       <c r="C259" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D259" t="n">
         <v>0</v>
       </c>
       <c r="E259" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F259" t="inlineStr">
         <is>
@@ -6807,13 +6807,13 @@
         <v>1</v>
       </c>
       <c r="C266" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="n">
         <v>0</v>
       </c>
       <c r="E266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F266" t="inlineStr">
         <is>
@@ -7167,13 +7167,13 @@
         <v>1</v>
       </c>
       <c r="C281" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D281" t="n">
         <v>0</v>
       </c>
       <c r="E281" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F281" t="inlineStr">
         <is>
@@ -7215,13 +7215,13 @@
         <v>1</v>
       </c>
       <c r="C283" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D283" t="n">
         <v>0</v>
       </c>
       <c r="E283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F283" t="inlineStr">
         <is>
@@ -7287,13 +7287,13 @@
         <v>1</v>
       </c>
       <c r="C286" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D286" t="n">
         <v>0</v>
       </c>
       <c r="E286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F286" t="inlineStr">
         <is>
@@ -7311,13 +7311,13 @@
         <v>1</v>
       </c>
       <c r="C287" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D287" t="n">
         <v>0</v>
       </c>
       <c r="E287" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F287" t="inlineStr">
         <is>
@@ -7719,13 +7719,13 @@
         <v>1</v>
       </c>
       <c r="C304" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D304" t="n">
         <v>0</v>
       </c>
       <c r="E304" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F304" t="inlineStr">
         <is>
@@ -7791,13 +7791,13 @@
         <v>1</v>
       </c>
       <c r="C307" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D307" t="n">
         <v>0</v>
       </c>
       <c r="E307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F307" t="inlineStr">
         <is>
@@ -7815,13 +7815,13 @@
         <v>1</v>
       </c>
       <c r="C308" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D308" t="n">
         <v>0</v>
       </c>
       <c r="E308" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F308" t="inlineStr">
         <is>
@@ -7887,13 +7887,13 @@
         <v>1</v>
       </c>
       <c r="C311" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D311" t="n">
         <v>0</v>
       </c>
       <c r="E311" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F311" t="inlineStr">
         <is>
@@ -7935,13 +7935,13 @@
         <v>1</v>
       </c>
       <c r="C313" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D313" t="n">
         <v>0</v>
       </c>
       <c r="E313" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F313" t="inlineStr">
         <is>
@@ -7959,13 +7959,13 @@
         <v>1</v>
       </c>
       <c r="C314" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D314" t="n">
         <v>0</v>
       </c>
       <c r="E314" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F314" t="inlineStr">
         <is>
@@ -8055,13 +8055,13 @@
         <v>1</v>
       </c>
       <c r="C318" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D318" t="n">
         <v>0</v>
       </c>
       <c r="E318" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F318" t="inlineStr">
         <is>
@@ -8415,13 +8415,13 @@
         <v>1</v>
       </c>
       <c r="C333" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D333" t="n">
         <v>0</v>
       </c>
       <c r="E333" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F333" t="inlineStr">
         <is>
@@ -8439,13 +8439,13 @@
         <v>1</v>
       </c>
       <c r="C334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="n">
         <v>0</v>
       </c>
       <c r="E334" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F334" t="inlineStr">
         <is>
@@ -8463,13 +8463,13 @@
         <v>1</v>
       </c>
       <c r="C335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="n">
         <v>0</v>
       </c>
       <c r="E335" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F335" t="inlineStr">
         <is>
@@ -8607,13 +8607,13 @@
         <v>1</v>
       </c>
       <c r="C341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D341" t="n">
         <v>0</v>
       </c>
       <c r="E341" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F341" t="inlineStr">
         <is>
@@ -8847,13 +8847,13 @@
         <v>1</v>
       </c>
       <c r="C351" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D351" t="n">
         <v>0</v>
       </c>
       <c r="E351" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F351" t="inlineStr">
         <is>
@@ -8895,13 +8895,13 @@
         <v>1</v>
       </c>
       <c r="C353" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D353" t="n">
         <v>0</v>
       </c>
       <c r="E353" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F353" t="inlineStr">
         <is>
@@ -8919,13 +8919,13 @@
         <v>1</v>
       </c>
       <c r="C354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" t="n">
         <v>0</v>
       </c>
       <c r="E354" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F354" t="inlineStr">
         <is>
@@ -9063,13 +9063,13 @@
         <v>1</v>
       </c>
       <c r="C360" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D360" t="n">
         <v>0</v>
       </c>
       <c r="E360" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F360" t="inlineStr">
         <is>
@@ -9663,13 +9663,13 @@
         <v>1</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="n">
         <v>0</v>
       </c>
       <c r="E385" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F385" t="inlineStr">
         <is>
@@ -9735,13 +9735,13 @@
         <v>1</v>
       </c>
       <c r="C388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="n">
         <v>0</v>
       </c>
       <c r="E388" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F388" t="inlineStr">
         <is>
@@ -9975,13 +9975,13 @@
         <v>1</v>
       </c>
       <c r="C398" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D398" t="n">
         <v>0</v>
       </c>
       <c r="E398" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F398" t="inlineStr">
         <is>
@@ -10023,13 +10023,13 @@
         <v>1</v>
       </c>
       <c r="C400" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D400" t="n">
         <v>0</v>
       </c>
       <c r="E400" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F400" t="inlineStr">
         <is>
@@ -10071,13 +10071,13 @@
         <v>1</v>
       </c>
       <c r="C402" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D402" t="n">
         <v>0</v>
       </c>
       <c r="E402" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F402" t="inlineStr">
         <is>
@@ -10095,13 +10095,13 @@
         <v>1</v>
       </c>
       <c r="C403" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D403" t="n">
         <v>0</v>
       </c>
       <c r="E403" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F403" t="inlineStr">
         <is>
@@ -10119,13 +10119,13 @@
         <v>1</v>
       </c>
       <c r="C404" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D404" t="n">
         <v>0</v>
       </c>
       <c r="E404" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F404" t="inlineStr">
         <is>
@@ -10335,13 +10335,13 @@
         <v>1</v>
       </c>
       <c r="C413" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D413" t="n">
         <v>0</v>
       </c>
       <c r="E413" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F413" t="inlineStr">
         <is>
@@ -10527,13 +10527,13 @@
         <v>1</v>
       </c>
       <c r="C421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="n">
         <v>0</v>
       </c>
       <c r="E421" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F421" t="inlineStr">
         <is>
@@ -10551,13 +10551,13 @@
         <v>1</v>
       </c>
       <c r="C422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="n">
         <v>0</v>
       </c>
       <c r="E422" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F422" t="inlineStr">
         <is>
@@ -10719,13 +10719,13 @@
         <v>1</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="n">
         <v>0</v>
       </c>
       <c r="E429" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F429" t="inlineStr">
         <is>
@@ -10887,13 +10887,13 @@
         <v>1</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="n">
         <v>0</v>
       </c>
       <c r="E436" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F436" t="inlineStr">
         <is>
@@ -11007,13 +11007,13 @@
         <v>1</v>
       </c>
       <c r="C441" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D441" t="n">
         <v>0</v>
       </c>
       <c r="E441" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F441" t="inlineStr">
         <is>
@@ -11199,13 +11199,13 @@
         <v>1</v>
       </c>
       <c r="C449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D449" t="n">
         <v>0</v>
       </c>
       <c r="E449" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F449" t="inlineStr">
         <is>
@@ -11247,13 +11247,13 @@
         <v>1</v>
       </c>
       <c r="C451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="n">
         <v>0</v>
       </c>
       <c r="E451" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F451" t="inlineStr">
         <is>
@@ -11607,13 +11607,13 @@
         <v>1</v>
       </c>
       <c r="C466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="n">
         <v>0</v>
       </c>
       <c r="E466" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F466" t="inlineStr">
         <is>
@@ -11631,13 +11631,13 @@
         <v>1</v>
       </c>
       <c r="C467" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D467" t="n">
         <v>0</v>
       </c>
       <c r="E467" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F467" t="inlineStr">
         <is>
@@ -11655,13 +11655,13 @@
         <v>1</v>
       </c>
       <c r="C468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="n">
         <v>0</v>
       </c>
       <c r="E468" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F468" t="inlineStr">
         <is>
@@ -11703,13 +11703,13 @@
         <v>1</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="n">
         <v>0</v>
       </c>
       <c r="E470" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F470" t="inlineStr">
         <is>
@@ -11895,13 +11895,13 @@
         <v>1</v>
       </c>
       <c r="C478" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D478" t="n">
         <v>0</v>
       </c>
       <c r="E478" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F478" t="inlineStr">
         <is>
@@ -11991,13 +11991,13 @@
         <v>1</v>
       </c>
       <c r="C482" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D482" t="n">
         <v>0</v>
       </c>
       <c r="E482" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F482" t="inlineStr">
         <is>
@@ -12015,13 +12015,13 @@
         <v>1</v>
       </c>
       <c r="C483" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D483" t="n">
         <v>0</v>
       </c>
       <c r="E483" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F483" t="inlineStr">
         <is>
@@ -12375,10 +12375,10 @@
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -12451,10 +12451,10 @@
         <v>1</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -12489,10 +12489,10 @@
         <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -12508,10 +12508,10 @@
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -12736,10 +12736,10 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -12907,10 +12907,10 @@
         <v>1</v>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
         <v>0</v>
@@ -12964,10 +12964,10 @@
         <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
@@ -13002,10 +13002,10 @@
         <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
         <v>0</v>
@@ -13116,10 +13116,10 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
         <v>0</v>
@@ -13306,10 +13306,10 @@
         <v>1</v>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E64" t="n">
         <v>0</v>
@@ -13458,10 +13458,10 @@
         <v>1</v>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E72" t="n">
         <v>0</v>
@@ -13515,10 +13515,10 @@
         <v>1</v>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
         <v>0</v>
@@ -13705,10 +13705,10 @@
         <v>1</v>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D85" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E85" t="n">
         <v>0</v>
@@ -13895,10 +13895,10 @@
         <v>1</v>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D95" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E95" t="n">
         <v>0</v>
@@ -13971,10 +13971,10 @@
         <v>1</v>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D99" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E99" t="n">
         <v>0</v>
@@ -14009,10 +14009,10 @@
         <v>1</v>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D101" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E101" t="n">
         <v>0</v>
@@ -14028,10 +14028,10 @@
         <v>1</v>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D102" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E102" t="n">
         <v>0</v>
@@ -14047,10 +14047,10 @@
         <v>1</v>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E103" t="n">
         <v>0</v>
@@ -14161,10 +14161,10 @@
         <v>1</v>
       </c>
       <c r="C109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E109" t="n">
         <v>0</v>
@@ -14180,10 +14180,10 @@
         <v>1</v>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E110" t="n">
         <v>0</v>
@@ -14294,10 +14294,10 @@
         <v>1</v>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D116" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E116" t="n">
         <v>0</v>
@@ -14351,10 +14351,10 @@
         <v>1</v>
       </c>
       <c r="C119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D119" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E119" t="n">
         <v>0</v>
@@ -14617,10 +14617,10 @@
         <v>1</v>
       </c>
       <c r="C133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D133" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E133" t="n">
         <v>0</v>
@@ -14788,10 +14788,10 @@
         <v>1</v>
       </c>
       <c r="C142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D142" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E142" t="n">
         <v>0</v>
@@ -14807,10 +14807,10 @@
         <v>1</v>
       </c>
       <c r="C143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D143" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E143" t="n">
         <v>0</v>
@@ -14997,10 +14997,10 @@
         <v>1</v>
       </c>
       <c r="C153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D153" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E153" t="n">
         <v>0</v>
@@ -15016,10 +15016,10 @@
         <v>1</v>
       </c>
       <c r="C154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D154" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E154" t="n">
         <v>0</v>
@@ -15035,10 +15035,10 @@
         <v>1</v>
       </c>
       <c r="C155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D155" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E155" t="n">
         <v>0</v>
@@ -15073,10 +15073,10 @@
         <v>1</v>
       </c>
       <c r="C157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D157" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E157" t="n">
         <v>0</v>
@@ -15111,10 +15111,10 @@
         <v>1</v>
       </c>
       <c r="C159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D159" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E159" t="n">
         <v>0</v>
@@ -15206,10 +15206,10 @@
         <v>1</v>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D164" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E164" t="n">
         <v>0</v>
@@ -15225,10 +15225,10 @@
         <v>1</v>
       </c>
       <c r="C165" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D165" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E165" t="n">
         <v>0</v>
@@ -15244,10 +15244,10 @@
         <v>1</v>
       </c>
       <c r="C166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D166" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E166" t="n">
         <v>0</v>
@@ -15396,10 +15396,10 @@
         <v>1</v>
       </c>
       <c r="C174" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D174" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E174" t="n">
         <v>0</v>
@@ -15510,10 +15510,10 @@
         <v>1</v>
       </c>
       <c r="C180" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D180" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E180" t="n">
         <v>0</v>
@@ -15548,10 +15548,10 @@
         <v>1</v>
       </c>
       <c r="C182" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D182" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E182" t="n">
         <v>0</v>
@@ -15624,10 +15624,10 @@
         <v>1</v>
       </c>
       <c r="C186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D186" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E186" t="n">
         <v>0</v>
@@ -15681,10 +15681,10 @@
         <v>1</v>
       </c>
       <c r="C189" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D189" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E189" t="n">
         <v>0</v>
@@ -15719,10 +15719,10 @@
         <v>1</v>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D191" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E191" t="n">
         <v>0</v>
@@ -15814,10 +15814,10 @@
         <v>1</v>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D196" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E196" t="n">
         <v>0</v>
@@ -15852,10 +15852,10 @@
         <v>1</v>
       </c>
       <c r="C198" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D198" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E198" t="n">
         <v>0</v>
@@ -16308,10 +16308,10 @@
         <v>1</v>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D222" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E222" t="n">
         <v>0</v>
@@ -16409,7 +16409,7 @@
         <v>1</v>
       </c>
       <c r="E227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="228">
@@ -16441,10 +16441,10 @@
         <v>1</v>
       </c>
       <c r="C229" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D229" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E229" t="n">
         <v>0</v>
@@ -16460,10 +16460,10 @@
         <v>1</v>
       </c>
       <c r="C230" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D230" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E230" t="n">
         <v>0</v>
@@ -16517,10 +16517,10 @@
         <v>1</v>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E233" t="n">
         <v>0</v>
@@ -16536,10 +16536,10 @@
         <v>1</v>
       </c>
       <c r="C234" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D234" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E234" t="n">
         <v>0</v>
@@ -16726,10 +16726,10 @@
         <v>1</v>
       </c>
       <c r="C244" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D244" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E244" t="n">
         <v>0</v>
@@ -16897,10 +16897,10 @@
         <v>1</v>
       </c>
       <c r="C253" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D253" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E253" t="n">
         <v>0</v>
@@ -17011,10 +17011,10 @@
         <v>1</v>
       </c>
       <c r="C259" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D259" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E259" t="n">
         <v>0</v>
@@ -17144,10 +17144,10 @@
         <v>1</v>
       </c>
       <c r="C266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E266" t="n">
         <v>0</v>
@@ -17429,10 +17429,10 @@
         <v>1</v>
       </c>
       <c r="C281" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D281" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E281" t="n">
         <v>0</v>
@@ -17467,10 +17467,10 @@
         <v>1</v>
       </c>
       <c r="C283" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D283" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E283" t="n">
         <v>0</v>
@@ -17524,10 +17524,10 @@
         <v>1</v>
       </c>
       <c r="C286" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D286" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E286" t="n">
         <v>0</v>
@@ -17543,10 +17543,10 @@
         <v>1</v>
       </c>
       <c r="C287" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D287" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E287" t="n">
         <v>0</v>
@@ -17866,10 +17866,10 @@
         <v>1</v>
       </c>
       <c r="C304" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D304" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E304" t="n">
         <v>0</v>
@@ -17923,10 +17923,10 @@
         <v>1</v>
       </c>
       <c r="C307" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D307" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E307" t="n">
         <v>0</v>
@@ -17942,10 +17942,10 @@
         <v>1</v>
       </c>
       <c r="C308" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D308" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E308" t="n">
         <v>0</v>
@@ -17999,10 +17999,10 @@
         <v>1</v>
       </c>
       <c r="C311" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D311" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E311" t="n">
         <v>0</v>
@@ -18037,10 +18037,10 @@
         <v>1</v>
       </c>
       <c r="C313" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D313" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E313" t="n">
         <v>0</v>
@@ -18056,10 +18056,10 @@
         <v>1</v>
       </c>
       <c r="C314" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D314" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E314" t="n">
         <v>0</v>
@@ -18132,10 +18132,10 @@
         <v>1</v>
       </c>
       <c r="C318" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D318" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E318" t="n">
         <v>0</v>
@@ -18417,10 +18417,10 @@
         <v>1</v>
       </c>
       <c r="C333" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D333" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E333" t="n">
         <v>0</v>
@@ -18436,10 +18436,10 @@
         <v>1</v>
       </c>
       <c r="C334" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E334" t="n">
         <v>0</v>
@@ -18455,10 +18455,10 @@
         <v>1</v>
       </c>
       <c r="C335" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E335" t="n">
         <v>0</v>
@@ -18569,10 +18569,10 @@
         <v>1</v>
       </c>
       <c r="C341" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E341" t="n">
         <v>0</v>
@@ -18759,10 +18759,10 @@
         <v>1</v>
       </c>
       <c r="C351" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D351" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E351" t="n">
         <v>0</v>
@@ -18797,10 +18797,10 @@
         <v>1</v>
       </c>
       <c r="C353" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D353" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E353" t="n">
         <v>0</v>
@@ -18816,10 +18816,10 @@
         <v>1</v>
       </c>
       <c r="C354" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E354" t="n">
         <v>0</v>
@@ -18930,10 +18930,10 @@
         <v>1</v>
       </c>
       <c r="C360" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D360" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E360" t="n">
         <v>0</v>
@@ -19405,10 +19405,10 @@
         <v>1</v>
       </c>
       <c r="C385" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E385" t="n">
         <v>0</v>
@@ -19462,10 +19462,10 @@
         <v>1</v>
       </c>
       <c r="C388" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D388" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E388" t="n">
         <v>0</v>
@@ -19652,10 +19652,10 @@
         <v>1</v>
       </c>
       <c r="C398" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D398" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E398" t="n">
         <v>0</v>
@@ -19690,10 +19690,10 @@
         <v>1</v>
       </c>
       <c r="C400" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D400" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E400" t="n">
         <v>0</v>
@@ -19728,10 +19728,10 @@
         <v>1</v>
       </c>
       <c r="C402" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D402" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E402" t="n">
         <v>0</v>
@@ -19747,10 +19747,10 @@
         <v>1</v>
       </c>
       <c r="C403" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D403" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E403" t="n">
         <v>0</v>
@@ -19766,10 +19766,10 @@
         <v>1</v>
       </c>
       <c r="C404" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D404" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E404" t="n">
         <v>0</v>
@@ -19937,10 +19937,10 @@
         <v>1</v>
       </c>
       <c r="C413" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D413" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E413" t="n">
         <v>0</v>
@@ -20089,10 +20089,10 @@
         <v>1</v>
       </c>
       <c r="C421" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E421" t="n">
         <v>0</v>
@@ -20108,10 +20108,10 @@
         <v>1</v>
       </c>
       <c r="C422" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E422" t="n">
         <v>0</v>
@@ -20241,10 +20241,10 @@
         <v>1</v>
       </c>
       <c r="C429" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E429" t="n">
         <v>0</v>
@@ -20374,10 +20374,10 @@
         <v>1</v>
       </c>
       <c r="C436" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E436" t="n">
         <v>0</v>
@@ -20469,10 +20469,10 @@
         <v>1</v>
       </c>
       <c r="C441" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D441" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E441" t="n">
         <v>0</v>
@@ -20621,10 +20621,10 @@
         <v>1</v>
       </c>
       <c r="C449" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E449" t="n">
         <v>0</v>
@@ -20659,10 +20659,10 @@
         <v>1</v>
       </c>
       <c r="C451" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E451" t="n">
         <v>0</v>
@@ -20944,10 +20944,10 @@
         <v>1</v>
       </c>
       <c r="C466" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D466" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E466" t="n">
         <v>0</v>
@@ -20963,10 +20963,10 @@
         <v>1</v>
       </c>
       <c r="C467" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D467" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E467" t="n">
         <v>0</v>
@@ -20982,10 +20982,10 @@
         <v>1</v>
       </c>
       <c r="C468" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D468" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E468" t="n">
         <v>0</v>
@@ -21020,10 +21020,10 @@
         <v>1</v>
       </c>
       <c r="C470" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E470" t="n">
         <v>0</v>
@@ -21172,10 +21172,10 @@
         <v>1</v>
       </c>
       <c r="C478" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D478" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E478" t="n">
         <v>0</v>
@@ -21248,10 +21248,10 @@
         <v>1</v>
       </c>
       <c r="C482" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D482" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E482" t="n">
         <v>0</v>
@@ -21267,10 +21267,10 @@
         <v>1</v>
       </c>
       <c r="C483" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D483" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E483" t="n">
         <v>0</v>

</xml_diff>